<commit_message>
Archive latest competition voice notes and scripts
Capture the current WonderEcho competition workflow and supporting scripts for rollback.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/项目总结/语音-WonderEchoPro/命令词播报词协议列表V3_中文_RAICOM比赛.xlsx
+++ b/项目总结/语音-WonderEchoPro/命令词播报词协议列表V3_中文_RAICOM比赛.xlsx
@@ -745,7 +745,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -824,10 +824,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1259,7 +1255,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J44"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
     <col width="19.3" customWidth="1" style="23" min="2" max="2"/>
@@ -1344,15 +1340,10 @@
       </c>
       <c r="I2" s="20" t="inlineStr">
         <is>
-          <t>控制性 协议01-0A不可改</t>
-        </is>
-      </c>
-      <c r="J2" s="21" t="inlineStr">
-        <is>
-          <t>协议固定
-不可更改</t>
-        </is>
-      </c>
+          <t>控制01-03勿改协议</t>
+        </is>
+      </c>
+      <c r="J2" s="21" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="24" t="n">
@@ -1460,447 +1451,214 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>增大音量</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>增大音量</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>增大音量</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>执行全自主运输任务</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>命令词</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>收到</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 04 00 FB</t>
-        </is>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 04 00 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>减小音量</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>减小音量</t>
-        </is>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>减小音量</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>小车收00 01=启动</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>开始全自主</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>命令词</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>收到</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="F7" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 05 00 FB</t>
-        </is>
-      </c>
-      <c r="G7" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 05 00 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>最大音量</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>最大音量</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>最大音量</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>开始运输</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>命令词</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>收到</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="F8" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 06 00 FB</t>
-        </is>
-      </c>
-      <c r="G8" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 06 00 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="24" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>中等音量</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>中等音量</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>中等音量</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F9" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 07 00 FB</t>
-        </is>
-      </c>
-      <c r="G9" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 07 00 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>最小音量</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>最小音量</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>最小音量</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F10" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 08 00 FB</t>
-        </is>
-      </c>
-      <c r="G10" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 08 00 FB</t>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>AA 55 00 01 FB</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>开启播报</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>开播报</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>开启播报</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F11" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 09 00 FB</t>
-        </is>
-      </c>
-      <c r="G11" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 09 00 FB</t>
-        </is>
-      </c>
+      <c r="A11" s="1" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>关闭播报</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>关播报</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
-        <is>
-          <t>关闭播报</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F12" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 0A 00 FB</t>
-        </is>
-      </c>
-      <c r="G12" s="25" t="inlineStr">
-        <is>
-          <t>AA 55 0A 00 FB</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>遥操作区任务已完成</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>播报语</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>遥操作区任务+已完成</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>被</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>AA 55 FF 01 FB</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>AA 55 FF 01 FB</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>小车发FF 01=播报</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="19" t="n"/>
       <c r="F14" s="19" t="n"/>
       <c r="G14" s="19" t="n"/>
-      <c r="I14" s="20" t="inlineStr">
-        <is>
-          <t>命令</t>
-        </is>
-      </c>
-      <c r="J14" s="22" t="inlineStr">
-        <is>
-          <t>00 xx
-(0x00开始)</t>
-        </is>
-      </c>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="22" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>执行全自主运输任务</t>
-        </is>
-      </c>
-      <c r="C15" s="28" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>收到</t>
-        </is>
-      </c>
-      <c r="E15" s="28" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
-      <c r="G15" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
-      <c r="I15" s="20" t="inlineStr">
-        <is>
-          <t>比赛启动 语义11 协议00 01</t>
-        </is>
-      </c>
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="I15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="29" t="inlineStr">
-        <is>
-          <t>开始全自主</t>
-        </is>
-      </c>
-      <c r="C16" s="28" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="D16" s="28" t="inlineStr">
-        <is>
-          <t>收到</t>
-        </is>
-      </c>
-      <c r="E16" s="28" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F16" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
-      <c r="G16" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>开始运输</t>
-        </is>
-      </c>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="inlineStr">
-        <is>
-          <t>收到</t>
-        </is>
-      </c>
-      <c r="E17" s="28" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F17" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
-      <c r="G17" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 01 FB</t>
-        </is>
-      </c>
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="29" t="inlineStr">
-        <is>
-          <t>停下</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
-        <is>
-          <t>已停止</t>
-        </is>
-      </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F18" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 02 FB</t>
-        </is>
-      </c>
-      <c r="G18" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 02 FB</t>
-        </is>
-      </c>
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>停止</t>
-        </is>
-      </c>
-      <c r="C19" s="28" t="inlineStr">
-        <is>
-          <t>命令词</t>
-        </is>
-      </c>
-      <c r="D19" s="28" t="inlineStr">
-        <is>
-          <t>已停止</t>
-        </is>
-      </c>
-      <c r="E19" s="28" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F19" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 02 FB</t>
-        </is>
-      </c>
-      <c r="G19" s="29" t="inlineStr">
-        <is>
-          <t>AA 55 00 02 FB</t>
-        </is>
-      </c>
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -1914,44 +1672,10 @@
       <c r="G21" s="19" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="n">
-        <v>13</v>
-      </c>
-      <c r="B22" s="31" t="inlineStr">
-        <is>
-          <t>遥操作区任务已完成</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr">
-        <is>
-          <t>播报语</t>
-        </is>
-      </c>
-      <c r="D22" s="30" t="inlineStr">
-        <is>
-          <t>遥操作区任务+已完成</t>
-        </is>
-      </c>
-      <c r="E22" s="30" t="inlineStr">
-        <is>
-          <t>被</t>
-        </is>
-      </c>
-      <c r="F22" s="31" t="inlineStr">
-        <is>
-          <t>AA 55 FF 01 FB</t>
-        </is>
-      </c>
-      <c r="G22" s="31" t="inlineStr">
-        <is>
-          <t>AA 55 FF 01 FB</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>比赛播报 被动发 FF 01</t>
-        </is>
-      </c>
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
@@ -2055,7 +1779,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B47"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="2.875" customWidth="1" style="23" min="1" max="1"/>
     <col width="103.875" customWidth="1" style="23" min="2" max="2"/>

</xml_diff>